<commit_message>
actualizando "productos" y "producto"
</commit_message>
<xml_diff>
--- a/data/lista_productos.xlsx
+++ b/data/lista_productos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DUOC\2 año\4to Semestre\FullStack 2\leveup\Level-Up\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DUOC\2 año\4to Semestre\FullStack 2\leveup\Level-Up\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F033BAF-23D8-496A-89F5-AD661262329F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C5F6907-8BA4-4A85-A215-8F2D6A2F8B97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>